<commit_message>
Refresh synthetic JWC timetable sample
Document that the JWC importer sample workbook is fully synthetic and contains no real institutional data. The end-to-end split test now points to the new README for fixture provenance, and the sample XLSX file was regenerated to match the documented synthetic dataset.
</commit_message>
<xml_diff>
--- a/backend/internal/importer/jwc/testdata/sample_timetable.xlsx
+++ b/backend/internal/importer/jwc/testdata/sample_timetable.xlsx
@@ -130,7 +130,7 @@
     <t>C00001</t>
   </si>
   <si>
-    <t>体育（4）</t>
+    <t>课程001</t>
   </si>
   <si>
     <t>专业A241,专业A242,专业A243,专业A244,专业B241,专业B242,专业B243,专业B244,专业C241,专业C242,专业C243,专业C244</t>
@@ -208,7 +208,7 @@
     <t>C00002</t>
   </si>
   <si>
-    <t>大学日语（2）</t>
+    <t>课程002</t>
   </si>
   <si>
     <t>教师001</t>
@@ -250,7 +250,7 @@
     <t>C00003</t>
   </si>
   <si>
-    <t>English for Academic Purpose 4 Direct Entry Program (EAP4DEP)</t>
+    <t>课程003</t>
   </si>
   <si>
     <t>专业P243</t>
@@ -295,7 +295,7 @@
     <t>C00004</t>
   </si>
   <si>
-    <t>机械基础</t>
+    <t>课程004</t>
   </si>
   <si>
     <t>专业F24,专业N24</t>
@@ -331,7 +331,7 @@
     <t>C00005</t>
   </si>
   <si>
-    <t>数据库原理及应用 (Database Principle and Application)</t>
+    <t>课程005</t>
   </si>
   <si>
     <t>专业Q243,专业Q244</t>
@@ -370,7 +370,7 @@
     <t>C00006</t>
   </si>
   <si>
-    <t>第二外语（1）</t>
+    <t>课程006</t>
   </si>
   <si>
     <t>专业R241,专业R242</t>
@@ -412,7 +412,7 @@
     <t>C00007</t>
   </si>
   <si>
-    <t>传感与检测技术</t>
+    <t>课程007</t>
   </si>
   <si>
     <t>专业S241,专业S242</t>
@@ -439,7 +439,7 @@
     <t>C00008</t>
   </si>
   <si>
-    <t>高分子化学与物理</t>
+    <t>课程008</t>
   </si>
   <si>
     <t>专业T241</t>
@@ -469,7 +469,7 @@
     <t>C00009</t>
   </si>
   <si>
-    <t>人际沟通理论</t>
+    <t>课程009</t>
   </si>
   <si>
     <t>专业U231,专业U232</t>
@@ -508,7 +508,7 @@
     <t>C00010</t>
   </si>
   <si>
-    <t>面向对象C++</t>
+    <t>课程010</t>
   </si>
   <si>
     <t>专业V241,专业V242,专业V243</t>
@@ -544,7 +544,7 @@
     <t>C00011</t>
   </si>
   <si>
-    <t>食品标准与法规</t>
+    <t>课程011</t>
   </si>
   <si>
     <t>专业M231,专业M232</t>
@@ -586,7 +586,7 @@
     <t>C00012</t>
   </si>
   <si>
-    <t>造纸工业自动控制原理与方法</t>
+    <t>课程012</t>
   </si>
   <si>
     <t>专业T231,专业T232,专业T233</t>
@@ -619,7 +619,7 @@
     <t>C00013</t>
   </si>
   <si>
-    <t>大学英语(2)</t>
+    <t>课程013</t>
   </si>
   <si>
     <t>专业B253,专业B254</t>
@@ -649,7 +649,7 @@
     <t>C00014</t>
   </si>
   <si>
-    <t>高等数学（二）</t>
+    <t>课程014</t>
   </si>
   <si>
     <t>专业W251,专业W252,专业W253,专业W254</t>
@@ -685,7 +685,7 @@
     <t>C00015</t>
   </si>
   <si>
-    <t>导览与解说</t>
+    <t>课程015</t>
   </si>
   <si>
     <t>专业U251,专业U252,专业U253</t>
@@ -715,7 +715,7 @@
     <t>C00016</t>
   </si>
   <si>
-    <t>数字电子技术基础</t>
+    <t>课程016</t>
   </si>
   <si>
     <t>专业B241,专业B242,专业B243,专业B244</t>
@@ -748,7 +748,7 @@
     <t>C00017</t>
   </si>
   <si>
-    <t>C语言程序设计</t>
+    <t>课程017</t>
   </si>
   <si>
     <t>专业X255,专业X256,专业X257,专业X258</t>
@@ -778,7 +778,7 @@
     <t>C00018</t>
   </si>
   <si>
-    <t>Web应用程序设计 (Web Application Development)</t>
+    <t>课程018</t>
   </si>
   <si>
     <t>专业Q231,专业Q232</t>
@@ -808,7 +808,7 @@
     <t>C00019</t>
   </si>
   <si>
-    <t>数字图像处理（双语）</t>
+    <t>课程019</t>
   </si>
   <si>
     <t>专业W241,专业W242,专业W243</t>
@@ -835,7 +835,7 @@
     <t>C00020</t>
   </si>
   <si>
-    <t>Python机器学习与大数据分析</t>
+    <t>课程020</t>
   </si>
   <si>
     <t>教师018</t>
@@ -865,7 +865,7 @@
     <t>C00021</t>
   </si>
   <si>
-    <t>概率论与数理统计</t>
+    <t>课程021</t>
   </si>
   <si>
     <t>专业P253,专业P254</t>
@@ -892,7 +892,7 @@
     <t>C00022</t>
   </si>
   <si>
-    <t>食品生物技术</t>
+    <t>课程022</t>
   </si>
   <si>
     <t>教师020</t>

</xml_diff>